<commit_message>
docs: add detailed instructions to each Excel sheet
Each of the 8 sheets now has a highlighted instruction block
with step-by-step guidance and risks to avoid.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/OpsFlow-Bootcamp-IESA-Flujo-Completo.xlsx
+++ b/docs/OpsFlow-Bootcamp-IESA-Flujo-Completo.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,8 +64,19 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000A1628"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000A1628"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -82,6 +93,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F0F2F5"/>
         <bgColor rgb="00F0F2F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8EDF5"/>
+        <bgColor rgb="00E8EDF5"/>
       </patternFill>
     </fill>
   </fills>
@@ -111,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -128,6 +145,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -494,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -923,10 +946,62 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>INSTRUCCIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="35" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>1. Esta hoja resume los 9 pasos del bootcamp. Cada módulo tiene su propia hoja con el formato de trabajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="35" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>2. La columna 'Tiempo sugerido' es orientativa — ajusta según el ritmo del grupo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="35" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>3. La columna 'Referencia' indica la fuente académica principal de cada módulo. Consúltalas para profundizar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="35" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>4. Los módulos están diseñados para seguirse en orden secuencial. Cada uno construye sobre el anterior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="35" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>5. En la plataforma OpsFlow cada módulo tiene una guía teórica completa antes del ejercicio práctico.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="9">
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A19:I19"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A18:I18"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A16:I16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -939,7 +1014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1261,10 +1336,78 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>INSTRUCCIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="35" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>1. Responde cada pregunta con el equipo, no solo una persona. El valor está en la discusión.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="35" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>2. Escala: 1 = No existe o es muy informal | 3 = Existe pero no es consistente | 5 = Sistemático y medido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="35" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>3. Si hay desacuerdo en el equipo sobre un puntaje, registra el comentario explicando las perspectivas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="35" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>4. Revisa el promedio final: Bajo (&lt;2.5) indica gaps críticos, Medio (2.5-3.8) hay base pero falta consistencia, Alto (≥3.8) el proceso es maduro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="35" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>5. Identifica las 2-3 categorías con puntaje más bajo — esas son tus focos de atención para los siguientes módulos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="35" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>6. RIESGO A EVITAR: No puntúes todo igual (todo 3). Si todas las respuestas son iguales, el diagnóstico no aporta información útil.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="35" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>7. En OpsFlow puedes usar el botón de IA para generar un análisis crítico que detecta contradicciones entre tus respuestas.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="11">
     <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A28:I28"/>
+    <mergeCell ref="A23:I23"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A27:I27"/>
+    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A24:I24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1277,7 +1420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1510,9 +1653,93 @@
       </c>
       <c r="D18" s="7" t="inlineStr"/>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>INSTRUCCIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="35" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>1. Lista TODOS los pasos del proceso en orden, desde que inicia la solicitud hasta que se entrega el resultado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="35" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>2. Tiempo de proceso (min) = minutos de TRABAJO ACTIVO en ese paso. NO incluye esperas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="35" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>3. Espera (h) = horas que pasan entre que termina este paso y empieza el siguiente. Incluye colas, aprobaciones, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="35" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>4. Retrabajo (%) = porcentaje de veces que hay que repetir o corregir algo en este paso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="35" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>5. ¿Agrega valor? = ¿El cliente final pagaría por este paso? Validaciones internas, aprobaciones y esperas NO agregan valor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="35" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>6. Lead time total = suma de todos los tiempos de proceso (convertidos a horas) + suma de todas las esperas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="35" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>7. Eficiencia de flujo = tiempo de valor / lead time total. En la mayoría de empresas está entre 1% y 5%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="35" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>8. RIESGO A EVITAR: Mapear el proceso ideal, no el real. El VSM debe reflejar lo que pasa HOY, incluyendo los workarounds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="35" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>9. No olvides los handoffs informales — si la coordinación es por WhatsApp, eso es un paso del proceso.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="12">
+    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A28:I28"/>
+    <mergeCell ref="A21:I21"/>
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A27:I27"/>
+    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A24:I24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1525,7 +1752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1737,9 +1964,85 @@
       <c r="G13" s="5" t="n"/>
       <c r="H13" s="5" t="n"/>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>INSTRUCCIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="35" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>1. Revisa cada paso del VSM y pregunta: ¿qué puede fallar aquí? ¿qué factores externos pueden afectarlo?</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="35" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>2. Tipos de riesgo sugeridos: Energía, Talento, Reposición, Gobierno, Proveedor externo, Disciplina comercial, Tecnología.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="35" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>3. Probabilidad: 1 = Raro | 2 = Poco probable | 3 = Posible | 4 = Probable | 5 = Casi seguro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="35" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>4. Impacto: 1 = Insignificante | 2 = Menor | 3 = Moderado | 4 = Mayor | 5 = Catastrófico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="35" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>5. Exposición = Probabilidad × Impacto. Se calcula automáticamente. Prioriza los de mayor exposición.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="35" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>6. Señales tempranas: ¿cómo sabrías que este riesgo se está activando ANTES de que se materialice?</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="35" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>7. Mitigaciones: acciones realistas con los recursos que tienes. No planes ideales que requieran inversión masiva.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="35" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>8. RIESGO A EVITAR: Normalizar riesgos. Que 'siempre hay microcortes' no significa que no sea un riesgo a gestionar.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="11">
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A24:I24"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A16:I16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1752,7 +2055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1972,9 +2275,93 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>INSTRUCCIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="35" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>1. Identifica cada problema operativo que genera costo: errores, esperas, retrabajos, quiebres, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="35" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>2. Frecuencia/semana: ¿cuántas veces por semana ocurre este problema? Usa datos reales si los tienes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="35" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>3. Minutos/evento: ¿cuánto tiempo se pierde cada vez que ocurre? Incluye el tiempo de todas las personas involucradas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="35" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>4. $/hora: costo hora laboral de quienes intervienen en corregir el problema. Salario mensual ÷ 160h es buena aproximación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="35" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>5. Unidades afectadas: si el problema causa pérdida de ventas, ¿cuántas unidades/pedidos se pierden por evento?</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="35" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>6. Margen/unidad: margen de contribución por cada unidad perdida. Ticket promedio × % margen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="35" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>7. Fórmula: Costo laboral mensual = (frecuencia × minutos / 60) × $/hora × 4.33 semanas/mes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="35" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>8. Fórmula: Costo total = Costo laboral + (Unidades × Margen × Frecuencia × 4.33).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="35" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>9. RIESGO A EVITAR: Inventar frecuencias sin datos. Mejor un estimado conservador que un número inflado.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="12">
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A14:I14"/>
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A16:I16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1987,7 +2374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2275,11 +2662,87 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>INSTRUCCIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="35" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>1. Lista todas las iniciativas que surgieron del diagnóstico, VSM, riesgos y desperdicio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="35" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>2. Para cada una, puntúa del 1 al 5 en cada dimensión. Usa criterio del equipo, no de una sola persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="35" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>3. Lead time: ¿cuánto reduce el tiempo total del proceso? | Económico: ¿cuánto dinero ahorra o genera?</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="35" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>4. Resiliencia: ¿hace al proceso más resistente a fallas? | Factibilidad: ¿se puede hacer en 30 días?</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="35" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>5. Esfuerzo (invertido): 1 = poco esfuerzo (mejor) | 5 = mucho esfuerzo. La fórmula invierte este valor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="35" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>6. Dep. externa (invertida): 1 = no depende de nadie (mejor) | 5 = depende de muchos. También se invierte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="35" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>7. Clasificación automática: ≥4.0 = Atacar ya | ≥3.2 = Diseñar | &lt;3.2 = Postergar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="35" customHeight="1">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>8. RIESGO A EVITAR: Puntuar todo alto para que todo salga 'Atacar ya'. Si no priorizas, no decidiste nada.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="13">
+    <mergeCell ref="A29:I29"/>
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A28:I28"/>
+    <mergeCell ref="A32:I32"/>
+    <mergeCell ref="A21:J21"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A27:I27"/>
+    <mergeCell ref="A30:I30"/>
     <mergeCell ref="A20:J20"/>
-    <mergeCell ref="A21:J21"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A24:I24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2292,7 +2755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2490,9 +2953,93 @@
       <c r="H13" s="5" t="n"/>
       <c r="I13" s="5" t="n"/>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>INSTRUCCIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="35" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>1. Solo incluye acciones de iniciativas clasificadas como 'Atacar ya'. Las demás van a un backlog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>2. Máximo 5 acciones. Mejor 5 bien ejecutadas que 15 a medias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>3. UN responsable por acción. Si 'todos' son responsables, nadie lo es.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="35" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>4. Métrica líder: el número que vas a medir para saber si la acción funcionó. Debe ser específica y medible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>5. Línea base: valor ACTUAL de la métrica (antes de la intervención).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>6. Meta: valor esperado al final de los 30 días. Sé ambicioso pero realista.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="35" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>7. Contingencia: ¿qué haces si la acción no funciona o se bloquea? Todo plan necesita un plan B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="35" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>8. RIESGO A EVITAR: Acciones vagas. 'Mejorar el proceso' NO es una acción. 'Implementar checklist de pedido con 5 campos obligatorios' SÍ lo es.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="35" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>9. Pon fechas realistas. No comprimas todo en la primera semana — distribuye la carga.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="12">
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A19:I19"/>
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A16:I16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2505,7 +3052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2679,9 +3226,101 @@
       <c r="G11" s="5" t="n"/>
       <c r="H11" s="5" t="n"/>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>INSTRUCCIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="35" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>1. Al final de CADA semana, registra las métricas. Si no mides, no sabes si estás mejorando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="35" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>2. Lead Time: tiempo promedio de punta a punta del proceso esa semana (en días).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="35" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>3. OTD/OTIF: porcentaje de entregas a tiempo y completas. La métrica de servicio al cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="35" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>4. Corregidos %: porcentaje de transacciones que requirieron corrección por errores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="35" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>5. Reprogramadas %: porcentaje de transacciones que se modificaron después de ingresadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>6. Retrabajo %: porcentaje de transacciones que requirieron re-procesamiento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>7. Avance plan %: porcentaje estimado de avance del plan de 30 días.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="35" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>8. ALERTA: Si una métrica empeora 2 semanas consecutivas, investiga la causa raíz antes de que sea crisis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="35" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>9. Notas: registra eventos inusuales (corte de energía, ausencia clave, cambio de prioridades) que expliquen variaciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="35" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>10. Compara siempre contra la línea base del plan — no contra la semana anterior solamente.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="13">
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A24:I24"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A16:I16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>